<commit_message>
Update text control and UI auto-generation
</commit_message>
<xml_diff>
--- a/Sample/Data/Locale/Locale.xlsx
+++ b/Sample/Data/Locale/Locale.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" r:id="Radcfdabd0e4049a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Languages" sheetId="12" r:id="Rad1a53f71dc240fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrs" sheetId="3" r:id="R322f73416dad4759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="Rdaedff3c5d7e4dca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="5" r:id="Rf807f37146c445a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="6" r:id="Ra7f063d981b2427c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="7" r:id="R694eed5dbb2e4215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="8" r:id="R48cc08f725b849b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="9" r:id="Rc12298a145934c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="10" r:id="R00db72dd3aa0487a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="11" r:id="R6abee059ce654c27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueNames" sheetId="13" r:id="Re2e92b9cb8974bc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueContents" sheetId="14" r:id="R70348ffda95c49ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI" sheetId="2" r:id="R1552b78e2a9c40f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Languages" sheetId="12" r:id="R5849768225c946e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attrs" sheetId="3" r:id="R879e9da0e63a48f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="4" r:id="R366338c37f4e444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enemies" sheetId="5" r:id="Rd1af22d17ef14718"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equips" sheetId="6" r:id="Ra46ba18b51034596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Classes" sheetId="7" r:id="R7cf7ca83fb454c46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="States" sheetId="8" r:id="Rcf557354a3a04076"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapNames" sheetId="9" r:id="R7f388f85fc824723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Specials" sheetId="10" r:id="R782bba78bfd241c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player" sheetId="11" r:id="R6b1a212ea74141f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueNames" sheetId="13" r:id="R49444da980f44773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DialogueContents" sheetId="14" r:id="Reeec8a35ba5e49e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1687,7 +1687,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -1695,6 +1695,9 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -2497,6 +2500,72 @@
         <x:v>157</x:v>
       </x:c>
     </x:row>
+    <x:row r="55" ht="32" customHeight="1">
+      <x:c r="A55" s="7" t="str">
+        <x:v>PLAYER_NAME_PROMPT</x:v>
+      </x:c>
+      <x:c r="B55" s="7" t="str">
+        <x:v>Enter a player name</x:v>
+      </x:c>
+      <x:c r="C55" s="7" t="str">
+        <x:v>请输入玩家名字</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="32" customHeight="1">
+      <x:c r="A56" s="7" t="str">
+        <x:v>PLAYER_NAME_EMPTY</x:v>
+      </x:c>
+      <x:c r="B56" s="7" t="str">
+        <x:v>Enter a non-empty name</x:v>
+      </x:c>
+      <x:c r="C56" s="7" t="str">
+        <x:v>名字不能为空</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="32" customHeight="1">
+      <x:c r="A57" s="7" t="str">
+        <x:v>PLAYER_NAME_TOO_LONG</x:v>
+      </x:c>
+      <x:c r="B57" s="7" t="str">
+        <x:v>Use 32 characters or fewer</x:v>
+      </x:c>
+      <x:c r="C57" s="7" t="str">
+        <x:v>名字最多 32 个字符</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="32" customHeight="1">
+      <x:c r="A58" s="7" t="str">
+        <x:v>PLAYER_NAME_CONFIRM</x:v>
+      </x:c>
+      <x:c r="B58" s="7" t="str">
+        <x:v>Confirm</x:v>
+      </x:c>
+      <x:c r="C58" s="7" t="str">
+        <x:v>确认</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="32" customHeight="1">
+      <x:c r="A59" s="7" t="str">
+        <x:v>PLAYER_NAME_CANCEL</x:v>
+      </x:c>
+      <x:c r="B59" s="7" t="str">
+        <x:v>Cancel</x:v>
+      </x:c>
+      <x:c r="C59" s="7" t="str">
+        <x:v>取消</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="32" customHeight="1">
+      <x:c r="A60" s="7" t="str">
+        <x:v>PLAYER_NAME_DONE</x:v>
+      </x:c>
+      <x:c r="B60" s="7" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="C60" s="7" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>